<commit_message>
feat: add RAGAS evaluation dashboard and export functionality for experimental benchmarking data
</commit_message>
<xml_diff>
--- a/eval/RAGAS_Results.xlsx
+++ b/eval/RAGAS_Results.xlsx
@@ -1,13 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RAGAS" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="RAGAS_TrungBinh" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="CauHoi_SWE301" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,13 +26,22 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F4E79"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -46,8 +56,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,171 +424,271 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B18"/>
+  <dimension ref="A1:C11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="19" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="3" max="3"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>Cấu hình</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>Giá trị</t>
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Chi so RAGAS</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Gia tri</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Y nghia</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Model sinh + judge</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>llama-3.3-70b-versatile (Groq)</t>
+          <t>faithfulness</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>0.917</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Cau tra loi bam ngu canh, it bia</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Embedding (answer_relevancy)</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>multilingual-e5-base (local)</t>
+          <t>answer_relevancy</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>0.953</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Cau tra loi sat cau hoi</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Môn / Số câu</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>SWE301 (Kiểm thử phần mềm) / 6</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Chỉ số RAGAS</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Giá trị trung bình</t>
-        </is>
-      </c>
-    </row>
+          <t>context_precision</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>0.917</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Ngu canh truy xuat lien quan</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>context_recall</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>1</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Ngu canh du de suy ra dap an</t>
+        </is>
+      </c>
+    </row>
+    <row r="6"/>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>faithfulness</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>0.917</v>
+          <t>Mon danh gia</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>SWE301</t>
+        </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>answer_relevancy</t>
+          <t>So cau</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.953</v>
+        <v>6</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>context_precision</t>
-        </is>
-      </c>
-      <c r="B9" t="n">
-        <v>0.917</v>
+          <t>Generator + Judge</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Groq llama-3.3-70b-versatile</t>
+        </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>context_recall</t>
-        </is>
-      </c>
-      <c r="B10" t="n">
+          <t>Embedding</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>multilingual-e5-base (local)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Nguon</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>eval/RAGAS_Results.md</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="70" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>STT</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Mon</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Cau hoi</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
         <v>1</v>
       </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Các câu đã đánh giá</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="n">
-        <v>1</v>
-      </c>
-      <c r="B13" t="inlineStr">
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>SWE301</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
         <is>
           <t>Kiểm thử phần mềm là gì / nhằm mục đích gì?</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" t="n">
+    <row r="3">
+      <c r="A3" t="n">
         <v>2</v>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>SWE301</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
         <is>
           <t>Quy trình kiểm thử được chia làm các cấp độ chính nào?</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" t="n">
+    <row r="4">
+      <c r="A4" t="n">
         <v>3</v>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>SWE301</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
         <is>
           <t>Kiểm thử đơn vị (Unit Testing) tập trung vào gì?</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" t="n">
+    <row r="5">
+      <c r="A5" t="n">
         <v>4</v>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>SWE301</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
         <is>
           <t>Ai thường viết Unit Testing?</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" t="n">
+    <row r="6">
+      <c r="A6" t="n">
         <v>5</v>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>SWE301</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
         <is>
           <t>Kiểm thử tích hợp (Integration Testing) kiểm tra điều gì?</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" t="n">
+    <row r="7">
+      <c r="A7" t="n">
         <v>6</v>
       </c>
-      <c r="B18" t="inlineStr">
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>SWE301</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
         <is>
           <t>Kiểm thử hệ thống (System Testing) đánh giá điều gì?</t>
         </is>

</xml_diff>